<commit_message>
Nhập tin hàng loạt: loại hình = mục cha, loại con vào ô đặc điểm — 3 cột mới loai_can_ho, loai_dat, loi_vao (khớp listingSpec); tệp mẫu + bảng tự kiểm Cowork (chủ dự án 29/10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/mau-nhap-tin-hang-loat.xlsx
+++ b/public/mau-nhap-tin-hang-loat.xlsx
@@ -722,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BB1"/>
+  <dimension ref="A1:BE1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.6328125" style="5" customWidth="1"/>
@@ -937,6 +937,21 @@
       <c r="BB1" s="6" t="s">
         <v>69</v>
       </c>
+      <c r="BC1" s="6" t="inlineStr">
+        <is>
+          <t>loai_can_ho</t>
+        </is>
+      </c>
+      <c r="BD1" s="6" t="inlineStr">
+        <is>
+          <t>loai_dat</t>
+        </is>
+      </c>
+      <c r="BE1" s="6" t="inlineStr">
+        <is>
+          <t>loi_vao</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>